<commit_message>
[서버] Stat 게임데이터 추가, EStatOp 추가, EStatGroup 추가, GameDataTable_Stat 에 Stat 데이터 검색로직 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Enum/GameEnum.xlsx
+++ b/Development/Common/GameData/Enum/GameEnum.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\Enum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C85D651-C285-4E75-821A-B1D17C6D98D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D863DB4-BC46-4220-9E54-69006D3DE503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enum" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="169">
   <si>
     <t>MonsterGrade</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -163,30 +174,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>AddHP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AddMP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AddAtk</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>HP추가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MP추가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>공격력추가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>ObjectType</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -237,6 +224,398 @@
   <si>
     <t>Fail</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatOp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Add</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>AddPct</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Amp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reduce</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Total</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>필수</t>
+  </si>
+  <si>
+    <t>합연산 (힘+)</t>
+  </si>
+  <si>
+    <t>합연산% (힘+%)</t>
+  </si>
+  <si>
+    <t>곱연산 (힘증폭)</t>
+  </si>
+  <si>
+    <t>점감곱연산 (힘감폭)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>총합</t>
+  </si>
+  <si>
+    <t>StatGroup</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Str</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Int</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PDef</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MDef</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MoveSpd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AtkSpd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CritRate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>힘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>지능</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>물리방어력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>마법방어력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이동속도</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>공격속도</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>크리티컬확률</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>StrAdd</t>
+  </si>
+  <si>
+    <t>IntAdd</t>
+  </si>
+  <si>
+    <t>HpAdd</t>
+  </si>
+  <si>
+    <t>MpAdd</t>
+  </si>
+  <si>
+    <t>PDefAdd</t>
+  </si>
+  <si>
+    <t>MDefAdd</t>
+  </si>
+  <si>
+    <t>MoveSpdAdd</t>
+  </si>
+  <si>
+    <t>AtkSpdAdd</t>
+  </si>
+  <si>
+    <t>CritRateAdd</t>
+  </si>
+  <si>
+    <t>StrAddPct</t>
+  </si>
+  <si>
+    <t>IntAddPct</t>
+  </si>
+  <si>
+    <t>HpAddPct</t>
+  </si>
+  <si>
+    <t>MpAddPct</t>
+  </si>
+  <si>
+    <t>PDefAddPct</t>
+  </si>
+  <si>
+    <t>MDefAddPct</t>
+  </si>
+  <si>
+    <t>MoveSpdAddPct</t>
+  </si>
+  <si>
+    <t>AtkSpdAddPct</t>
+  </si>
+  <si>
+    <t>CritRateAddPct</t>
+  </si>
+  <si>
+    <t>StrAmp</t>
+  </si>
+  <si>
+    <t>IntAmp</t>
+  </si>
+  <si>
+    <t>HpAmp</t>
+  </si>
+  <si>
+    <t>MpAmp</t>
+  </si>
+  <si>
+    <t>PDefAmp</t>
+  </si>
+  <si>
+    <t>MDefAmp</t>
+  </si>
+  <si>
+    <t>MoveSpdAmp</t>
+  </si>
+  <si>
+    <t>AtkSpdAmp</t>
+  </si>
+  <si>
+    <t>CritRateAmp</t>
+  </si>
+  <si>
+    <t>StrReduce</t>
+  </si>
+  <si>
+    <t>IntReduce</t>
+  </si>
+  <si>
+    <t>HpReduce</t>
+  </si>
+  <si>
+    <t>MpReduce</t>
+  </si>
+  <si>
+    <t>PDefReduce</t>
+  </si>
+  <si>
+    <t>MDefReduce</t>
+  </si>
+  <si>
+    <t>MoveSpdReduce</t>
+  </si>
+  <si>
+    <t>AtkSpdReduce</t>
+  </si>
+  <si>
+    <t>CritRateReduce</t>
+  </si>
+  <si>
+    <t>StrTotal</t>
+  </si>
+  <si>
+    <t>IntTotal</t>
+  </si>
+  <si>
+    <t>HpTotal</t>
+  </si>
+  <si>
+    <t>MpTotal</t>
+  </si>
+  <si>
+    <t>PDefTotal</t>
+  </si>
+  <si>
+    <t>MDefTotal</t>
+  </si>
+  <si>
+    <t>MoveSpdTotal</t>
+  </si>
+  <si>
+    <t>AtkSpdTotal</t>
+  </si>
+  <si>
+    <t>CritRateTotal</t>
+  </si>
+  <si>
+    <t>힘+</t>
+  </si>
+  <si>
+    <t>힘+%</t>
+  </si>
+  <si>
+    <t>힘증폭</t>
+  </si>
+  <si>
+    <t>힘감폭</t>
+  </si>
+  <si>
+    <t>힘총합</t>
+  </si>
+  <si>
+    <t>지능+</t>
+  </si>
+  <si>
+    <t>지능+%</t>
+  </si>
+  <si>
+    <t>지능증폭</t>
+  </si>
+  <si>
+    <t>지능감폭</t>
+  </si>
+  <si>
+    <t>지능총합</t>
+  </si>
+  <si>
+    <t>HP+</t>
+  </si>
+  <si>
+    <t>HP+%</t>
+  </si>
+  <si>
+    <t>HP증폭</t>
+  </si>
+  <si>
+    <t>HP감폭</t>
+  </si>
+  <si>
+    <t>HP총합</t>
+  </si>
+  <si>
+    <t>MP+</t>
+  </si>
+  <si>
+    <t>MP+%</t>
+  </si>
+  <si>
+    <t>MP증폭</t>
+  </si>
+  <si>
+    <t>MP감폭</t>
+  </si>
+  <si>
+    <t>MP총합</t>
+  </si>
+  <si>
+    <t>물리방어력+</t>
+  </si>
+  <si>
+    <t>물리방어력+%</t>
+  </si>
+  <si>
+    <t>물리방어력증폭</t>
+  </si>
+  <si>
+    <t>물리방어력감폭</t>
+  </si>
+  <si>
+    <t>물리방어력총합</t>
+  </si>
+  <si>
+    <t>마법방어력+</t>
+  </si>
+  <si>
+    <t>마법방어력+%</t>
+  </si>
+  <si>
+    <t>마법방어력증폭</t>
+  </si>
+  <si>
+    <t>마법방어력감폭</t>
+  </si>
+  <si>
+    <t>마법방어력총합</t>
+  </si>
+  <si>
+    <t>이동속도+</t>
+  </si>
+  <si>
+    <t>이동속도+%</t>
+  </si>
+  <si>
+    <t>이동속도증폭</t>
+  </si>
+  <si>
+    <t>이동속도감폭</t>
+  </si>
+  <si>
+    <t>이동속도총합</t>
+  </si>
+  <si>
+    <t>공격속도+</t>
+  </si>
+  <si>
+    <t>공격속도+%</t>
+  </si>
+  <si>
+    <t>공격속도증폭</t>
+  </si>
+  <si>
+    <t>공격속도감폭</t>
+  </si>
+  <si>
+    <t>공격속도총합</t>
+  </si>
+  <si>
+    <t>치명타확률+</t>
+  </si>
+  <si>
+    <t>치명타확률+%</t>
+  </si>
+  <si>
+    <t>치명타확률증폭</t>
+  </si>
+  <si>
+    <t>치명타확률감폭</t>
+  </si>
+  <si>
+    <t>치명타확률총합</t>
   </si>
 </sst>
 </file>
@@ -312,7 +691,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -322,6 +701,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -603,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.5" style="1" customWidth="1"/>
@@ -790,13 +1172,13 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -861,10 +1243,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C15" s="1">
         <v>0</v>
@@ -875,183 +1257,1175 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C17" s="1">
         <v>2</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1">
         <v>3</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C19" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>30</v>
+        <v>37</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C20" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C21" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C22" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C23" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
+      </c>
+      <c r="E23" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="1">
-        <v>0</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>30</v>
+      <c r="E24" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C25" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E25" s="1" t="s">
         <v>50</v>
+      </c>
+      <c r="E25" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="1">
+        <v>3</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="1">
+        <v>4</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="1">
+        <v>5</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="1">
+        <v>0</v>
+      </c>
+      <c r="D29" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="1">
+        <v>1</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="1">
+        <v>2</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="1">
+        <v>3</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" s="1">
+        <v>4</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="1">
+        <v>5</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="1">
         <v>6</v>
       </c>
-      <c r="C26" s="1">
+      <c r="D35" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="1">
+        <v>7</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37" s="1">
+        <v>8</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="1">
+        <v>9</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="1">
+        <v>0</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" s="1">
         <v>2</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>51</v>
+      <c r="D41" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F41" s="4"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42" s="1">
+        <v>3</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43" s="1">
+        <v>4</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C44" s="1">
+        <v>5</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C45" s="1">
+        <v>6</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="1">
+        <v>7</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F46" s="4"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C47" s="1">
+        <v>8</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48" s="1">
+        <v>9</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C49" s="1">
+        <v>10</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C50" s="1">
+        <v>11</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C51" s="1">
+        <v>12</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F51" s="4"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C52" s="1">
+        <v>13</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53" s="1">
+        <v>14</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C54" s="1">
+        <v>15</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C55" s="1">
+        <v>16</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" s="1">
+        <v>17</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F56" s="4"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57" s="1">
+        <v>18</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C58" s="1">
+        <v>19</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="1">
+        <v>20</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" s="1">
+        <v>21</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C61" s="1">
+        <v>22</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F61" s="4"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="1">
+        <v>23</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" s="1">
+        <v>24</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C64" s="1">
+        <v>25</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C65" s="1">
+        <v>26</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C66" s="1">
+        <v>27</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F66" s="4"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C67" s="1">
+        <v>28</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C68" s="1">
+        <v>29</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C69" s="1">
+        <v>30</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C70" s="1">
+        <v>31</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71" s="1">
+        <v>32</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F71" s="4"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C72" s="1">
+        <v>33</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C73" s="1">
+        <v>34</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C74" s="1">
+        <v>35</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C75" s="1">
+        <v>36</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C76" s="1">
+        <v>37</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F76" s="4"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C77" s="1">
+        <v>38</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C78" s="1">
+        <v>39</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C79" s="1">
+        <v>40</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="1">
+        <v>41</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C81" s="1">
+        <v>42</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="F81" s="4"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C82" s="1">
+        <v>43</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C83" s="1">
+        <v>44</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C84" s="1">
+        <v>45</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[서버] Buff 게임데이터 추가, EBuffCategory, EBuffStackPolicy, EPeriodicEffect 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Enum/GameEnum.xlsx
+++ b/Development/Common/GameData/Enum/GameEnum.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\Enum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204534C3-EBD9-4A37-B28D-BCCBF65ADB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93583AB-17EE-4503-AF0D-F870ED581CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5355" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38865" yWindow="5910" windowWidth="27360" windowHeight="14340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enum" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="239">
   <si>
     <t>MonsterGrade</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -765,6 +765,83 @@
   <si>
     <t>효과의 발생 기준 위치</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BuffCategory</t>
+  </si>
+  <si>
+    <t>BuffCategory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Buff</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BuffStackPolicy</t>
+  </si>
+  <si>
+    <t>PeriodicEffect</t>
+  </si>
+  <si>
+    <t>Debuff</t>
+  </si>
+  <si>
+    <t>Refresh</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>Ignore</t>
+  </si>
+  <si>
+    <t>DamageHp</t>
+  </si>
+  <si>
+    <t>HealHp</t>
+  </si>
+  <si>
+    <t>이로운효과</t>
+  </si>
+  <si>
+    <t>해로운효과</t>
+  </si>
+  <si>
+    <t>디스펠 대상</t>
+  </si>
+  <si>
+    <t>시간갱신</t>
+  </si>
+  <si>
+    <t>재적용 시 지속시간만 리셋</t>
+  </si>
+  <si>
+    <t>스택증가</t>
+  </si>
+  <si>
+    <t>재적용 시 스택+1 (MaxStack까지)</t>
+  </si>
+  <si>
+    <t>무시</t>
+  </si>
+  <si>
+    <t>이미 있으면 무시</t>
+  </si>
+  <si>
+    <t>주기효과 없음</t>
+  </si>
+  <si>
+    <t>HP감소</t>
+  </si>
+  <si>
+    <t>DoT</t>
+  </si>
+  <si>
+    <t>HP회복</t>
+  </si>
+  <si>
+    <t>HoT</t>
   </si>
 </sst>
 </file>
@@ -1134,7 +1211,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.5" style="1" customWidth="1"/>
@@ -2955,6 +3032,188 @@
         <v>212</v>
       </c>
     </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C107" s="1">
+        <v>0</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C108" s="1">
+        <v>1</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C109" s="1">
+        <v>2</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C110" s="1">
+        <v>0</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C111" s="1">
+        <v>1</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C112" s="1">
+        <v>2</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C113" s="1">
+        <v>3</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C114" s="1">
+        <v>0</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C115" s="1">
+        <v>1</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C116" s="1">
+        <v>2</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[데이터] Spawner, SpawnGroup 데이터 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Enum/GameEnum.xlsx
+++ b/Development/Common/GameData/Enum/GameEnum.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\Enum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D949E5D-813E-4DA0-9EE1-7E73EA4D8B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E727D6E9-16B5-426C-A3E7-B486EDF821A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="5355" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enum" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="298">
   <si>
     <t>Enum 이름</t>
   </si>
@@ -913,6 +913,54 @@
   </si>
   <si>
     <t>몬스터 AI 종류</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SpawnActivation</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>스폰 활성화 모드</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Always</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>항상</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>항상 밀도 유지</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PlayerProximity</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>근접 활성</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>플레이어 근접 시만</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Manual</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>수동</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stage 스크립트에서 ActivateSpawner 등으로 활성화시킴</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1338,7 +1386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.75" style="1" customWidth="1"/>
@@ -3399,6 +3447,69 @@
         <v>284</v>
       </c>
     </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A114" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D114" s="1">
+        <v>1</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A115" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D115" s="1">
+        <v>2</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D116" s="1">
+        <v>3</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>297</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="E1:E111" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
[서버] ObjectType::User 를 ObjectType::Character로 변경
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Enum/GameEnum.xlsx
+++ b/Development/Common/GameData/Enum/GameEnum.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\MMOGameServerProject\Development\Common\GameData\Enum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFC1C08-27D8-4541-BC28-38A489CA0AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC18D725-F76D-41B2-8425-6E31E1C15D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5355" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enum" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Enum!$E$1:$E$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Enum!$E$1:$E$113</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="313">
   <si>
     <t>Enum 이름</t>
   </si>
@@ -957,18 +957,38 @@
   </si>
   <si>
     <t>상호작용 시 지정 스테이지/위치로 이동(무스크립트)</t>
+  </si>
+  <si>
+    <t>Character</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>캐릭터</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>NPC</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1076,46 +1096,49 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1398,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.75" style="1" customWidth="1"/>
@@ -1669,11 +1692,11 @@
       <c r="D15" s="7">
         <v>1</v>
       </c>
-      <c r="E15" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>10</v>
+      <c r="E15" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1746,19 +1769,19 @@
     </row>
     <row r="20" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="7">
-        <v>1</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>49</v>
+        <v>6</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1769,30 +1792,30 @@
         <v>8</v>
       </c>
       <c r="D21" s="7">
+        <v>1</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="7">
         <v>2</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E22" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F22" s="7" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D22" s="4">
-        <v>1</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1803,13 +1826,13 @@
         <v>53</v>
       </c>
       <c r="D23" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F23" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1820,13 +1843,13 @@
         <v>53</v>
       </c>
       <c r="D24" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1837,13 +1860,13 @@
         <v>53</v>
       </c>
       <c r="D25" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1854,30 +1877,30 @@
         <v>53</v>
       </c>
       <c r="D26" s="4">
+        <v>4</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="4">
         <v>5</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E27" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F27" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="D27" s="7">
-        <v>1</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1888,13 +1911,13 @@
         <v>53</v>
       </c>
       <c r="D28" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1905,13 +1928,13 @@
         <v>53</v>
       </c>
       <c r="D29" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1922,13 +1945,13 @@
         <v>53</v>
       </c>
       <c r="D30" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1939,13 +1962,13 @@
         <v>53</v>
       </c>
       <c r="D31" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1956,13 +1979,13 @@
         <v>53</v>
       </c>
       <c r="D32" s="7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1973,13 +1996,13 @@
         <v>53</v>
       </c>
       <c r="D33" s="7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -1990,13 +2013,13 @@
         <v>53</v>
       </c>
       <c r="D34" s="7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -2007,30 +2030,30 @@
         <v>53</v>
       </c>
       <c r="D35" s="7">
+        <v>8</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="7">
         <v>9</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E36" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="F36" s="7" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D36" s="4">
-        <v>1</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2041,15 +2064,14 @@
         <v>53</v>
       </c>
       <c r="D37" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="G37" s="8"/>
+        <v>84</v>
+      </c>
     </row>
     <row r="38" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
@@ -2059,14 +2081,15 @@
         <v>53</v>
       </c>
       <c r="D38" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>88</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
@@ -2076,13 +2099,13 @@
         <v>53</v>
       </c>
       <c r="D39" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2093,13 +2116,13 @@
         <v>53</v>
       </c>
       <c r="D40" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2110,13 +2133,13 @@
         <v>53</v>
       </c>
       <c r="D41" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2127,15 +2150,14 @@
         <v>53</v>
       </c>
       <c r="D42" s="4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="G42" s="8"/>
+        <v>94</v>
+      </c>
     </row>
     <row r="43" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
@@ -2145,14 +2167,15 @@
         <v>53</v>
       </c>
       <c r="D43" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>98</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="G43" s="8"/>
     </row>
     <row r="44" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
@@ -2162,13 +2185,13 @@
         <v>53</v>
       </c>
       <c r="D44" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="45" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2179,13 +2202,13 @@
         <v>53</v>
       </c>
       <c r="D45" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="46" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2196,13 +2219,13 @@
         <v>53</v>
       </c>
       <c r="D46" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2213,15 +2236,14 @@
         <v>53</v>
       </c>
       <c r="D47" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="G47" s="8"/>
+        <v>104</v>
+      </c>
     </row>
     <row r="48" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
@@ -2231,14 +2253,15 @@
         <v>53</v>
       </c>
       <c r="D48" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>108</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="G48" s="8"/>
     </row>
     <row r="49" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
@@ -2248,13 +2271,13 @@
         <v>53</v>
       </c>
       <c r="D49" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2265,13 +2288,13 @@
         <v>53</v>
       </c>
       <c r="D50" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2282,13 +2305,13 @@
         <v>53</v>
       </c>
       <c r="D51" s="4">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2299,15 +2322,14 @@
         <v>53</v>
       </c>
       <c r="D52" s="4">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="G52" s="8"/>
+        <v>114</v>
+      </c>
     </row>
     <row r="53" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
@@ -2317,14 +2339,15 @@
         <v>53</v>
       </c>
       <c r="D53" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>118</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G53" s="8"/>
     </row>
     <row r="54" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
@@ -2334,13 +2357,13 @@
         <v>53</v>
       </c>
       <c r="D54" s="4">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="55" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2351,13 +2374,13 @@
         <v>53</v>
       </c>
       <c r="D55" s="4">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2368,13 +2391,13 @@
         <v>53</v>
       </c>
       <c r="D56" s="4">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2385,15 +2408,14 @@
         <v>53</v>
       </c>
       <c r="D57" s="4">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="G57" s="8"/>
+        <v>124</v>
+      </c>
     </row>
     <row r="58" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
@@ -2403,14 +2425,15 @@
         <v>53</v>
       </c>
       <c r="D58" s="4">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>128</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="G58" s="8"/>
     </row>
     <row r="59" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
@@ -2420,13 +2443,13 @@
         <v>53</v>
       </c>
       <c r="D59" s="4">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="60" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2437,13 +2460,13 @@
         <v>53</v>
       </c>
       <c r="D60" s="4">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2454,13 +2477,13 @@
         <v>53</v>
       </c>
       <c r="D61" s="4">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="62" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2471,15 +2494,14 @@
         <v>53</v>
       </c>
       <c r="D62" s="4">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="G62" s="8"/>
+        <v>134</v>
+      </c>
     </row>
     <row r="63" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
@@ -2489,14 +2511,15 @@
         <v>53</v>
       </c>
       <c r="D63" s="4">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>138</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="G63" s="8"/>
     </row>
     <row r="64" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
@@ -2506,13 +2529,13 @@
         <v>53</v>
       </c>
       <c r="D64" s="4">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="65" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2523,13 +2546,13 @@
         <v>53</v>
       </c>
       <c r="D65" s="4">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="66" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2540,13 +2563,13 @@
         <v>53</v>
       </c>
       <c r="D66" s="4">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="67" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2557,15 +2580,14 @@
         <v>53</v>
       </c>
       <c r="D67" s="4">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="G67" s="8"/>
+        <v>144</v>
+      </c>
     </row>
     <row r="68" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
@@ -2575,14 +2597,15 @@
         <v>53</v>
       </c>
       <c r="D68" s="4">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>148</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="G68" s="8"/>
     </row>
     <row r="69" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
@@ -2592,13 +2615,13 @@
         <v>53</v>
       </c>
       <c r="D69" s="4">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="70" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2609,13 +2632,13 @@
         <v>53</v>
       </c>
       <c r="D70" s="4">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="71" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2626,13 +2649,13 @@
         <v>53</v>
       </c>
       <c r="D71" s="4">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="72" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2643,15 +2666,14 @@
         <v>53</v>
       </c>
       <c r="D72" s="4">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="G72" s="8"/>
+        <v>154</v>
+      </c>
     </row>
     <row r="73" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
@@ -2661,14 +2683,15 @@
         <v>53</v>
       </c>
       <c r="D73" s="4">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>158</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="G73" s="8"/>
     </row>
     <row r="74" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
@@ -2678,13 +2701,13 @@
         <v>53</v>
       </c>
       <c r="D74" s="4">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="75" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2695,13 +2718,13 @@
         <v>53</v>
       </c>
       <c r="D75" s="4">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="76" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2712,13 +2735,13 @@
         <v>53</v>
       </c>
       <c r="D76" s="4">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2729,15 +2752,14 @@
         <v>53</v>
       </c>
       <c r="D77" s="4">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G77" s="8"/>
+        <v>164</v>
+      </c>
     </row>
     <row r="78" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
@@ -2747,14 +2769,15 @@
         <v>53</v>
       </c>
       <c r="D78" s="4">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>168</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="G78" s="8"/>
     </row>
     <row r="79" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
@@ -2764,13 +2787,13 @@
         <v>53</v>
       </c>
       <c r="D79" s="4">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="80" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2781,33 +2804,30 @@
         <v>53</v>
       </c>
       <c r="D80" s="4">
+        <v>44</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D81" s="4">
         <v>45</v>
       </c>
-      <c r="E80" s="4" t="s">
+      <c r="E81" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="F80" s="4" t="s">
+      <c r="F81" s="4" t="s">
         <v>172</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="C81" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D81" s="7">
-        <v>1</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="F81" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="G81" s="7" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="82" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -2818,16 +2838,16 @@
         <v>174</v>
       </c>
       <c r="D82" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G82" s="7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="83" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -2838,53 +2858,56 @@
         <v>174</v>
       </c>
       <c r="D83" s="7">
+        <v>2</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="F83" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D84" s="7">
         <v>3</v>
       </c>
-      <c r="E83" s="5" t="s">
+      <c r="E84" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="F83" s="5" t="s">
+      <c r="F84" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="G83" s="7" t="s">
+      <c r="G84" s="7" t="s">
         <v>183</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>184</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="D84" s="4">
-        <v>1</v>
-      </c>
-      <c r="E84" t="s">
-        <v>186</v>
-      </c>
-      <c r="F84" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="85" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>184</v>
       </c>
+      <c r="B85" s="4" t="s">
+        <v>185</v>
+      </c>
       <c r="C85" s="4" t="s">
         <v>174</v>
       </c>
       <c r="D85" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E85" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F85" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2895,13 +2918,13 @@
         <v>174</v>
       </c>
       <c r="D86" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E86" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F86" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="87" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2912,51 +2935,50 @@
         <v>174</v>
       </c>
       <c r="D87" s="4">
+        <v>3</v>
+      </c>
+      <c r="E87" t="s">
+        <v>190</v>
+      </c>
+      <c r="F87" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>184</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D88" s="4">
         <v>4</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E88" t="s">
         <v>192</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F88" t="s">
         <v>193</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B88" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C88" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D88" s="7">
-        <v>1</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="F88" s="5" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="89" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="B89" s="5"/>
+      <c r="B89" s="7" t="s">
+        <v>195</v>
+      </c>
       <c r="C89" s="7" t="s">
         <v>174</v>
       </c>
       <c r="D89" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="90" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -2968,223 +2990,223 @@
         <v>174</v>
       </c>
       <c r="D90" s="7">
+        <v>2</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B91" s="5"/>
+      <c r="C91" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D91" s="7">
         <v>3</v>
       </c>
-      <c r="E90" s="5" t="s">
+      <c r="E91" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="F90" s="5" t="s">
+      <c r="F91" s="5" t="s">
         <v>201</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>202</v>
-      </c>
-      <c r="B91" t="s">
-        <v>203</v>
-      </c>
-      <c r="C91" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="D91" s="4">
-        <v>1</v>
-      </c>
-      <c r="E91" t="s">
-        <v>204</v>
-      </c>
-      <c r="F91" t="s">
-        <v>205</v>
-      </c>
-      <c r="G91" s="4" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="92" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>202</v>
       </c>
+      <c r="B92" t="s">
+        <v>203</v>
+      </c>
       <c r="C92" s="4" t="s">
         <v>174</v>
       </c>
       <c r="D92" s="4">
+        <v>1</v>
+      </c>
+      <c r="E92" t="s">
+        <v>204</v>
+      </c>
+      <c r="F92" t="s">
+        <v>205</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>202</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D93" s="4">
         <v>2</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E93" t="s">
         <v>207</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F93" t="s">
         <v>208</v>
       </c>
-      <c r="G92" s="4" t="s">
+      <c r="G93" s="4" t="s">
         <v>209</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B93" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="C93" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D93" s="7">
-        <v>1</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="F93" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G93" s="7" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="94" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="B94" s="5"/>
+      <c r="B94" s="7" t="s">
+        <v>211</v>
+      </c>
       <c r="C94" s="7" t="s">
         <v>174</v>
       </c>
       <c r="D94" s="7">
+        <v>1</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B95" s="5"/>
+      <c r="C95" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D95" s="7">
         <v>2</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="E95" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="F94" s="5" t="s">
+      <c r="F95" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G94" s="7" t="s">
+      <c r="G95" s="7" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="95" spans="1:7" s="4" customFormat="1" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="B95" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="D95" s="4">
-        <v>1</v>
-      </c>
-      <c r="E95" t="s">
-        <v>220</v>
-      </c>
-      <c r="F95" t="s">
-        <v>221</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" s="4" customFormat="1" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="B96" s="9"/>
+      <c r="B96" s="10" t="s">
+        <v>219</v>
+      </c>
       <c r="C96" s="4" t="s">
         <v>174</v>
       </c>
       <c r="D96" s="4">
+        <v>1</v>
+      </c>
+      <c r="E96" t="s">
+        <v>220</v>
+      </c>
+      <c r="F96" t="s">
+        <v>221</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="B97" s="9"/>
+      <c r="C97" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D97" s="4">
         <v>2</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E97" t="s">
         <v>223</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F97" t="s">
         <v>224</v>
       </c>
-      <c r="G96" s="4" t="s">
+      <c r="G97" s="4" t="s">
         <v>225</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="B97" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="C97" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D97" s="7">
-        <v>1</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="F97" s="5" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="98" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B98" s="5"/>
+      <c r="B98" s="7" t="s">
+        <v>227</v>
+      </c>
       <c r="C98" s="7" t="s">
         <v>174</v>
       </c>
       <c r="D98" s="7">
+        <v>1</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="B99" s="5"/>
+      <c r="C99" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D99" s="7">
         <v>2</v>
       </c>
-      <c r="E98" s="5" t="s">
+      <c r="E99" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="F98" s="5" t="s">
+      <c r="F99" s="5" t="s">
         <v>231</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="D99" s="4">
-        <v>1</v>
-      </c>
-      <c r="E99" t="s">
-        <v>234</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="G99" s="4" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="100" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A100" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B100" s="9"/>
+      <c r="B100" s="4" t="s">
+        <v>233</v>
+      </c>
       <c r="C100" s="4" t="s">
         <v>174</v>
       </c>
       <c r="D100" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E100" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>238</v>
+        <v>235</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="101" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3196,30 +3218,31 @@
         <v>174</v>
       </c>
       <c r="D101" s="4">
+        <v>2</v>
+      </c>
+      <c r="E101" t="s">
+        <v>237</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B102" s="9"/>
+      <c r="C102" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D102" s="4">
         <v>3</v>
       </c>
-      <c r="E101" t="s">
+      <c r="E102" t="s">
         <v>239</v>
       </c>
-      <c r="F101" s="4" t="s">
+      <c r="F102" s="4" t="s">
         <v>240</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="C102" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="D102" s="7">
-        <v>1</v>
-      </c>
-      <c r="E102" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="F102" s="7" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="103" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
@@ -3230,36 +3253,33 @@
         <v>242</v>
       </c>
       <c r="D103" s="7">
+        <v>1</v>
+      </c>
+      <c r="E103" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="F103" s="7" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D104" s="7">
         <v>2</v>
       </c>
-      <c r="E103" s="7" t="s">
+      <c r="E104" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="F103" s="7" t="s">
+      <c r="F104" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="G103" s="7" t="s">
+      <c r="G104" s="7" t="s">
         <v>246</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="C104" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="D104" s="4">
-        <v>1</v>
-      </c>
-      <c r="E104" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="F104" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="G104" s="4" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="105" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3270,16 +3290,16 @@
         <v>242</v>
       </c>
       <c r="D105" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G105" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="106" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3290,79 +3310,79 @@
         <v>242</v>
       </c>
       <c r="D106" s="4">
+        <v>2</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="F106" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="G106" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D107" s="4">
         <v>3</v>
       </c>
-      <c r="E106" s="4" t="s">
+      <c r="E107" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="F106" s="4" t="s">
+      <c r="F107" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="G106" s="4" t="s">
+      <c r="G107" s="4" t="s">
         <v>256</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="B107" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="C107" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="D107" s="7">
-        <v>1</v>
-      </c>
-      <c r="E107" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="F107" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="G107" s="7" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="108" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A108" s="7" t="s">
         <v>257</v>
       </c>
+      <c r="B108" s="7" t="s">
+        <v>258</v>
+      </c>
       <c r="C108" s="7" t="s">
         <v>242</v>
       </c>
       <c r="D108" s="7">
+        <v>1</v>
+      </c>
+      <c r="E108" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="F108" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="G108" s="7" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D109" s="7">
         <v>2</v>
       </c>
-      <c r="E108" s="7" t="s">
+      <c r="E109" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="F108" s="7" t="s">
+      <c r="F109" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="G108" s="7" t="s">
+      <c r="G109" s="7" t="s">
         <v>264</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
-        <v>265</v>
-      </c>
-      <c r="C109" t="s">
-        <v>30</v>
-      </c>
-      <c r="D109" s="4">
-        <v>1</v>
-      </c>
-      <c r="E109" t="s">
-        <v>266</v>
-      </c>
-      <c r="F109" t="s">
-        <v>267</v>
-      </c>
-      <c r="G109" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="110" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3373,16 +3393,16 @@
         <v>30</v>
       </c>
       <c r="D110" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E110" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="F110" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="G110" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="111" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3393,16 +3413,16 @@
         <v>30</v>
       </c>
       <c r="D111" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E111" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F111" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G111" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="112" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3413,102 +3433,102 @@
         <v>30</v>
       </c>
       <c r="D112" s="4">
+        <v>3</v>
+      </c>
+      <c r="E112" t="s">
+        <v>272</v>
+      </c>
+      <c r="F112" t="s">
+        <v>273</v>
+      </c>
+      <c r="G112" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>265</v>
+      </c>
+      <c r="C113" t="s">
+        <v>30</v>
+      </c>
+      <c r="D113" s="4">
         <v>4</v>
       </c>
-      <c r="E112" t="s">
+      <c r="E113" t="s">
         <v>275</v>
       </c>
-      <c r="F112" t="s">
+      <c r="F113" t="s">
         <v>276</v>
       </c>
-      <c r="G112" t="s">
+      <c r="G113" t="s">
         <v>277</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="B113" s="12" t="s">
-        <v>279</v>
-      </c>
-      <c r="C113" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D113" s="13">
-        <v>1</v>
-      </c>
-      <c r="E113" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="F113" s="12" t="s">
-        <v>281</v>
-      </c>
-      <c r="G113" s="12" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="114" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A114" s="12" t="s">
         <v>278</v>
       </c>
+      <c r="B114" s="12" t="s">
+        <v>279</v>
+      </c>
       <c r="C114" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D114" s="13">
+        <v>1</v>
+      </c>
+      <c r="E114" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="F114" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="G114" s="12" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="C115" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D115" s="13">
         <v>2</v>
       </c>
-      <c r="E114" s="12" t="s">
+      <c r="E115" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="F114" s="12" t="s">
+      <c r="F115" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="G114" s="12" t="s">
+      <c r="G115" s="12" t="s">
         <v>285</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A115" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="B115" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D115" s="1">
-        <v>1</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="G115" s="1" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>286</v>
       </c>
+      <c r="B116" s="1" t="s">
+        <v>287</v>
+      </c>
       <c r="C116" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D116" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.3">
@@ -3519,87 +3539,107 @@
         <v>11</v>
       </c>
       <c r="D117" s="1">
+        <v>2</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A118" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D118" s="1">
         <v>3</v>
       </c>
-      <c r="E117" s="1" t="s">
+      <c r="E118" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="F117" s="1" t="s">
+      <c r="F118" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="G117" s="1" t="s">
+      <c r="G118" s="1" t="s">
         <v>296</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="12" t="s">
-        <v>297</v>
-      </c>
-      <c r="B118" s="12" t="s">
-        <v>298</v>
-      </c>
-      <c r="C118" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D118" s="13">
-        <v>1</v>
-      </c>
-      <c r="E118" s="12" t="s">
-        <v>299</v>
-      </c>
-      <c r="F118" s="12" t="s">
-        <v>300</v>
-      </c>
-      <c r="G118" s="12" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="119" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A119" s="12" t="s">
         <v>297</v>
       </c>
+      <c r="B119" s="12" t="s">
+        <v>298</v>
+      </c>
       <c r="C119" s="12" t="s">
         <v>41</v>
       </c>
       <c r="D119" s="13">
+        <v>1</v>
+      </c>
+      <c r="E119" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="F119" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="G119" s="12" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="C120" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D120" s="13">
         <v>2</v>
       </c>
-      <c r="E119" s="12" t="s">
+      <c r="E120" s="12" t="s">
         <v>302</v>
       </c>
-      <c r="F119" s="12" t="s">
+      <c r="F120" s="12" t="s">
         <v>303</v>
       </c>
-      <c r="G119" s="12" t="s">
+      <c r="G120" s="12" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
         <v>305</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B121" t="s">
         <v>306</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C121" t="s">
         <v>41</v>
       </c>
-      <c r="D120" s="4">
+      <c r="D121" s="4">
         <v>1</v>
       </c>
-      <c r="E120" t="s">
+      <c r="E121" t="s">
         <v>307</v>
       </c>
-      <c r="F120" t="s">
+      <c r="F121" t="s">
         <v>308</v>
       </c>
-      <c r="G120" t="s">
+      <c r="G121" t="s">
         <v>309</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="E1:E112" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <autoFilter ref="E1:E113" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>